<commit_message>
Added entry for Jill Beckmann
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I123"/>
+  <dimension ref="A1:H124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,11 +473,6 @@
           <t>Authorized Drivers</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Unique ID</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -497,7 +492,7 @@
         <v>45595</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>45596</v>
+        <v>45596.99930555555</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -510,9 +505,6 @@
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="n">
-        <v>24</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -532,7 +524,7 @@
         <v>45574</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45575</v>
+        <v>45575.99930555555</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -545,9 +537,6 @@
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="n">
-        <v>27</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -567,7 +556,7 @@
         <v>45593</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>45593</v>
+        <v>45593.99930555555</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -580,9 +569,6 @@
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="n">
-        <v>23</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -602,7 +588,7 @@
         <v>45560</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45561</v>
+        <v>45561.99930555555</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -615,9 +601,6 @@
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -637,7 +620,7 @@
         <v>45546</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>45547</v>
+        <v>45547.99930555555</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -650,9 +633,6 @@
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="n">
-        <v>21</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -672,22 +652,15 @@
         <v>45421</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>45421</v>
+        <v>45421.99930555555</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>268 - 2017 Ford F-150, Silver(6 Seats)</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -707,7 +680,7 @@
         <v>45567</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45568</v>
+        <v>45568.99930555555</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -720,9 +693,6 @@
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="n">
-        <v>19</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -742,22 +712,15 @@
         <v>45539</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45540</v>
+        <v>45540.99930555555</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>268 - 2017 Ford F-150, Silver(6 Seats)</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="n">
-        <v>18</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -777,7 +740,7 @@
         <v>45553</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45554</v>
+        <v>45554.99930555555</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -790,9 +753,6 @@
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="n">
-        <v>17</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -812,7 +772,7 @@
         <v>45551</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45551</v>
+        <v>45551.99930555555</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -825,9 +785,6 @@
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="n">
-        <v>16</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -847,7 +804,7 @@
         <v>45558</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45558</v>
+        <v>45558.99930555555</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -860,9 +817,6 @@
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -882,7 +836,7 @@
         <v>45432</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>45538</v>
+        <v>45538.99930555555</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -895,9 +849,6 @@
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -917,7 +868,7 @@
         <v>45600</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45600</v>
+        <v>45600.99930555555</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -930,9 +881,6 @@
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -952,22 +900,15 @@
         <v>45401</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45402</v>
+        <v>45402.99930555555</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>268 - 2017 Ford F-150, Silver(6 Seats)</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="n">
-        <v>13</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -987,7 +928,7 @@
         <v>45576</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>45576</v>
+        <v>45576.99930555555</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1000,9 +941,6 @@
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="n">
-        <v>29</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1022,7 +960,7 @@
         <v>45579</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>45579</v>
+        <v>45579.99930555555</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1035,9 +973,6 @@
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1057,7 +992,7 @@
         <v>45588</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45589</v>
+        <v>45589.99930555555</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1070,9 +1005,6 @@
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>31</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1092,7 +1024,7 @@
         <v>45581</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>45582</v>
+        <v>45582.99930555555</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1105,9 +1037,6 @@
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="n">
-        <v>28</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1127,7 +1056,7 @@
         <v>45572</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>45572</v>
+        <v>45572.99930555555</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1140,9 +1069,6 @@
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1162,7 +1088,7 @@
         <v>45581</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>45585</v>
+        <v>45585.99930555555</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1175,9 +1101,6 @@
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="n">
-        <v>32</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1197,7 +1120,7 @@
         <v>45588</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>45588</v>
+        <v>45588.99930555555</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1210,9 +1133,6 @@
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="n">
-        <v>33</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1232,22 +1152,15 @@
         <v>45554</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>45556</v>
+        <v>45556.99930555555</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>310 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="n">
-        <v>34</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1267,7 +1180,7 @@
         <v>45600</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>45600</v>
+        <v>45600.99930555555</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1280,9 +1193,6 @@
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="n">
-        <v>35</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1302,7 +1212,7 @@
         <v>45627</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>45635</v>
+        <v>45635.99930555555</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1315,9 +1225,6 @@
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="n">
-        <v>36</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1337,7 +1244,7 @@
         <v>45605</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>45610</v>
+        <v>45610.99930555555</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1350,9 +1257,6 @@
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" t="n">
-        <v>37</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1372,22 +1276,15 @@
         <v>45637</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>45642</v>
+        <v>45642.99930555555</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>310 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
-      <c r="I27" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1407,7 +1304,7 @@
         <v>45594</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>45595</v>
+        <v>45595.99930555555</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1420,9 +1317,6 @@
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="n">
-        <v>39</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1442,22 +1336,15 @@
         <v>45660</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>45670</v>
+        <v>45670.99930555555</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>310 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1477,7 +1364,7 @@
         <v>45608</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>45608</v>
+        <v>45608.99930555555</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1490,9 +1377,6 @@
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="n">
-        <v>49</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1512,7 +1396,7 @@
         <v>45611</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>45611</v>
+        <v>45611.99930555555</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1525,9 +1409,6 @@
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="n">
-        <v>47</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1547,7 +1428,7 @@
         <v>45603</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>45604</v>
+        <v>45604.99930555555</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1560,9 +1441,6 @@
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
-      <c r="I32" t="n">
-        <v>46</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1582,22 +1460,15 @@
         <v>45597</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>45598</v>
+        <v>45598.99930555555</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
           <t>321 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
-      <c r="I33" t="n">
-        <v>45</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1617,22 +1488,15 @@
         <v>45548</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>45554</v>
+        <v>45554.99930555555</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
           <t>321 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="n">
-        <v>44</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1652,22 +1516,15 @@
         <v>45562</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>45564</v>
+        <v>45564.99930555555</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
           <t>321 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="n">
-        <v>43</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1687,22 +1544,15 @@
         <v>45568</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>45568</v>
+        <v>45568.99930555555</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>321 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="n">
-        <v>42</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1722,22 +1572,15 @@
         <v>45589</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>45593</v>
+        <v>45593.99930555555</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>321 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="n">
-        <v>41</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1757,7 +1600,7 @@
         <v>45581</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>45587</v>
+        <v>45587.99930555555</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1770,9 +1613,6 @@
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
-      <c r="I38" t="n">
-        <v>40</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1792,7 +1632,7 @@
         <v>45627</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>45748</v>
+        <v>45748.99930555555</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -1808,9 +1648,6 @@
         <is>
           <t>Emory Ellis</t>
         </is>
-      </c>
-      <c r="I39" t="n">
-        <v>48</v>
       </c>
     </row>
     <row r="40">
@@ -1831,22 +1668,15 @@
         <v>45552</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>45554</v>
+        <v>45554.99930555555</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
           <t>325 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1866,22 +1696,15 @@
         <v>45566</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>45568</v>
+        <v>45568.99930555555</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>325 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="n">
-        <v>56</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1901,7 +1724,7 @@
         <v>45586</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>45610</v>
+        <v>45610.99930555555</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -1914,9 +1737,6 @@
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="n">
-        <v>55</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1936,22 +1756,15 @@
         <v>45573</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>45575</v>
+        <v>45575.99930555555</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>325 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="n">
-        <v>54</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1971,22 +1784,15 @@
         <v>45559</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>45561</v>
+        <v>45561.99930555555</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>325 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
-      <c r="I44" t="n">
-        <v>53</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2006,22 +1812,15 @@
         <v>45580</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>45582</v>
+        <v>45582.99930555555</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>325 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="n">
-        <v>52</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2041,22 +1840,15 @@
         <v>45545</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>45547</v>
+        <v>45547.99930555555</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
           <t>325 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="n">
-        <v>51</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2076,7 +1868,7 @@
         <v>45642</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>45643</v>
+        <v>45643.99930555555</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2092,9 +1884,6 @@
         <is>
           <t>Keven Griffen</t>
         </is>
-      </c>
-      <c r="I47" t="n">
-        <v>62</v>
       </c>
     </row>
     <row r="48">
@@ -2115,22 +1904,15 @@
         <v>45595</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>45595</v>
+        <v>45595.99930555555</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
-      <c r="I48" t="n">
-        <v>58</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2150,22 +1932,15 @@
         <v>45588</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>45588</v>
+        <v>45588.99930555555</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="n">
-        <v>57</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2185,22 +1960,15 @@
         <v>45565</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>45567</v>
+        <v>45567.99930555555</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
-      <c r="I50" t="n">
-        <v>59</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2220,22 +1988,15 @@
         <v>45576</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>45576</v>
+        <v>45576.99930555555</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="n">
-        <v>61</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2255,7 +2016,7 @@
         <v>45581</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>45583</v>
+        <v>45583.99930555555</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2268,9 +2029,6 @@
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
-      <c r="I52" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2290,25 +2048,18 @@
         <v>45667</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>45667</v>
+        <v>45667.99930555555</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>Jacob Shelly</t>
         </is>
-      </c>
-      <c r="I53" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="54">
@@ -2329,25 +2080,18 @@
         <v>45667</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>45667</v>
+        <v>45667.99930555555</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>Jacob Shelly</t>
         </is>
-      </c>
-      <c r="I54" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="55">
@@ -2368,25 +2112,18 @@
         <v>45667</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>45667</v>
+        <v>45667.99930555555</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>Jacob Shelly</t>
         </is>
-      </c>
-      <c r="I55" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="56">
@@ -2407,25 +2144,18 @@
         <v>45667</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>45667</v>
+        <v>45667.99930555555</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>Jacob Shelly</t>
         </is>
-      </c>
-      <c r="I56" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="57">
@@ -2446,25 +2176,18 @@
         <v>45667</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>45667</v>
+        <v>45667.99930555555</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>Jacob Shelly</t>
         </is>
-      </c>
-      <c r="I57" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="58">
@@ -2485,25 +2208,18 @@
         <v>45667</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>45667</v>
+        <v>45667.99930555555</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>Jacob Shelly</t>
         </is>
-      </c>
-      <c r="I58" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="59">
@@ -2524,25 +2240,18 @@
         <v>45667</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>45667</v>
+        <v>45667.99930555555</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>Jacob Shelly</t>
         </is>
-      </c>
-      <c r="I59" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="60">
@@ -2563,25 +2272,18 @@
         <v>45667</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>45667</v>
+        <v>45667.99930555555</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>Jacob Shelly</t>
         </is>
-      </c>
-      <c r="I60" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="61">
@@ -2602,25 +2304,18 @@
         <v>45667</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>45667</v>
+        <v>45667.99930555555</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
           <t>329 - Chevy Trail Boss, White</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>Jacob Shelly</t>
         </is>
-      </c>
-      <c r="I61" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="62">
@@ -2641,25 +2336,18 @@
         <v>45631</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>45643</v>
+        <v>45643.99930555555</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
           <t>330 - Toyota Camry</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>Sierra Jech</t>
         </is>
-      </c>
-      <c r="I62" t="n">
-        <v>64</v>
       </c>
     </row>
     <row r="63">
@@ -2680,7 +2368,7 @@
         <v>45642</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>45642</v>
+        <v>45642.99930555555</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -2696,9 +2384,6 @@
         <is>
           <t>{Colin Whitehead}{Max yusen}{Cole Brant}</t>
         </is>
-      </c>
-      <c r="I63" t="n">
-        <v>72</v>
       </c>
     </row>
     <row r="64">
@@ -2719,7 +2404,7 @@
         <v>45572</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>45576</v>
+        <v>45576.99930555555</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -2735,9 +2420,6 @@
         <is>
           <t>Wade Axup</t>
         </is>
-      </c>
-      <c r="I64" t="n">
-        <v>73</v>
       </c>
     </row>
     <row r="65">
@@ -2758,7 +2440,7 @@
         <v>45613</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>45619</v>
+        <v>45619.99930555555</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -2774,9 +2456,6 @@
         <is>
           <t>Wade Axup</t>
         </is>
-      </c>
-      <c r="I65" t="n">
-        <v>71</v>
       </c>
     </row>
     <row r="66">
@@ -2797,7 +2476,7 @@
         <v>45629</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>45633</v>
+        <v>45633.99930555555</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -2813,9 +2492,6 @@
         <is>
           <t>Wade Axup</t>
         </is>
-      </c>
-      <c r="I66" t="n">
-        <v>70</v>
       </c>
     </row>
     <row r="67">
@@ -2836,22 +2512,15 @@
         <v>45611</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>45611</v>
+        <v>45611.99930555555</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
           <t>331- 2024  Toyota Sienna Hybrid, White (8 seats)</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
-      <c r="I67" t="n">
-        <v>69</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2871,25 +2540,18 @@
         <v>45481</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>45490</v>
+        <v>45490.99930555555</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
           <t>331- 2024  Toyota Sienna Hybrid, White (8 seats)</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>Jasmine Anenberg</t>
         </is>
-      </c>
-      <c r="I68" t="n">
-        <v>68</v>
       </c>
     </row>
     <row r="69">
@@ -2910,7 +2572,7 @@
         <v>45605</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>45609</v>
+        <v>45609.99930555555</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -2923,9 +2585,6 @@
         </is>
       </c>
       <c r="H69" t="inlineStr"/>
-      <c r="I69" t="n">
-        <v>67</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2945,7 +2604,7 @@
         <v>45534</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>45553</v>
+        <v>45553.99930555555</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -2958,9 +2617,6 @@
         </is>
       </c>
       <c r="H70" t="inlineStr"/>
-      <c r="I70" t="n">
-        <v>66</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2980,25 +2636,18 @@
         <v>45503</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>45503</v>
+        <v>45503.99930555555</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
           <t>331- 2024  Toyota Sienna Hybrid, White (8 seats)</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>Shay Levine</t>
         </is>
-      </c>
-      <c r="I71" t="n">
-        <v>65</v>
       </c>
     </row>
     <row r="72">
@@ -3019,22 +2668,15 @@
         <v>45568</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>45568</v>
+        <v>45568.99930555555</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
           <t>331- 2024  Toyota Sienna Hybrid, White (8 seats)</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
-      <c r="I72" t="n">
-        <v>63</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3054,7 +2696,7 @@
         <v>45525</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>45525</v>
+        <v>45525.99930555555</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -3067,9 +2709,6 @@
         </is>
       </c>
       <c r="H73" t="inlineStr"/>
-      <c r="I73" t="n">
-        <v>81</v>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3089,7 +2728,7 @@
         <v>45509</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>45514</v>
+        <v>45514.99930555555</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -3105,9 +2744,6 @@
         <is>
           <t>Matthew Voorhees</t>
         </is>
-      </c>
-      <c r="I74" t="n">
-        <v>80</v>
       </c>
     </row>
     <row r="75">
@@ -3128,7 +2764,7 @@
         <v>45517</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>45518</v>
+        <v>45518.99930555555</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -3144,9 +2780,6 @@
         <is>
           <t>Salli Dymond</t>
         </is>
-      </c>
-      <c r="I75" t="n">
-        <v>79</v>
       </c>
     </row>
     <row r="76">
@@ -3167,7 +2800,7 @@
         <v>45439</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>45445</v>
+        <v>45445.99930555555</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -3180,9 +2813,6 @@
         </is>
       </c>
       <c r="H76" t="inlineStr"/>
-      <c r="I76" t="n">
-        <v>78</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3202,7 +2832,7 @@
         <v>45432</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>45434</v>
+        <v>45434.99930555555</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -3215,9 +2845,6 @@
         </is>
       </c>
       <c r="H77" t="inlineStr"/>
-      <c r="I77" t="n">
-        <v>77</v>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3237,7 +2864,7 @@
         <v>45453</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>45477</v>
+        <v>45477.99930555555</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -3250,9 +2877,6 @@
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
-      <c r="I78" t="n">
-        <v>76</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3272,7 +2896,7 @@
         <v>45478</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>45506</v>
+        <v>45506.99930555555</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -3285,9 +2909,6 @@
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
-      <c r="I79" t="n">
-        <v>75</v>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3307,22 +2928,15 @@
         <v>45555</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>45555</v>
+        <v>45555.99930555555</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
           <t>332 - 2009 Dodge Dakota, White (5 Seats)</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr"/>
-      <c r="I80" t="n">
-        <v>74</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3342,22 +2956,15 @@
         <v>45421</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>45421</v>
+        <v>45421.99930555555</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
           <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr"/>
-      <c r="I81" t="n">
-        <v>91</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3377,7 +2984,7 @@
         <v>45444</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>45536</v>
+        <v>45536.99930555555</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -3390,9 +2997,6 @@
         </is>
       </c>
       <c r="H82" t="inlineStr"/>
-      <c r="I82" t="n">
-        <v>89</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3412,22 +3016,15 @@
         <v>45639</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>45647</v>
+        <v>45647.99930555555</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
           <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr"/>
-      <c r="I83" t="n">
-        <v>90</v>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3447,22 +3044,15 @@
         <v>45422</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>45427</v>
+        <v>45427.99930555555</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
           <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr"/>
-      <c r="I84" t="n">
-        <v>88</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -3482,22 +3072,15 @@
         <v>45617</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>45623</v>
+        <v>45623.99930555555</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
           <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr"/>
-      <c r="I85" t="n">
-        <v>87</v>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -3517,22 +3100,15 @@
         <v>45627</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>45636</v>
+        <v>45636.99930555555</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
           <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
-      <c r="I86" t="n">
-        <v>85</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -3552,22 +3128,15 @@
         <v>45602</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>45608</v>
+        <v>45608.99930555555</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
           <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr"/>
-      <c r="I87" t="n">
-        <v>86</v>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -3587,22 +3156,15 @@
         <v>45401</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>45402</v>
+        <v>45402.99930555555</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
           <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr"/>
-      <c r="I88" t="n">
-        <v>83</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -3622,7 +3184,7 @@
         <v>45541</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>45571</v>
+        <v>45571.99930555555</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -3635,9 +3197,6 @@
         </is>
       </c>
       <c r="H89" t="inlineStr"/>
-      <c r="I89" t="n">
-        <v>82</v>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -3657,25 +3216,18 @@
         <v>45627</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>45688</v>
+        <v>45688.99930555555</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
           <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>Keven Griffen</t>
         </is>
-      </c>
-      <c r="I90" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="91">
@@ -3696,22 +3248,15 @@
         <v>45432</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>45433</v>
+        <v>45433.99930555555</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
           <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
-      <c r="I91" t="n">
-        <v>84</v>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -3731,22 +3276,15 @@
         <v>45403</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>45423</v>
+        <v>45423.99930555555</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
           <t>338 - 2012 Nissan Titan, White (5 Seats)</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr"/>
-      <c r="I92" t="n">
-        <v>97</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -3766,7 +3304,7 @@
         <v>45425</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>45474</v>
+        <v>45474.99930555555</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -3779,9 +3317,6 @@
         </is>
       </c>
       <c r="H93" t="inlineStr"/>
-      <c r="I93" t="n">
-        <v>96</v>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3801,7 +3336,7 @@
         <v>45475</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>45565</v>
+        <v>45565.99930555555</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -3814,9 +3349,6 @@
         </is>
       </c>
       <c r="H94" t="inlineStr"/>
-      <c r="I94" t="n">
-        <v>98</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -3836,7 +3368,7 @@
         <v>45581</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>45587</v>
+        <v>45587.99930555555</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -3849,9 +3381,6 @@
         </is>
       </c>
       <c r="H95" t="inlineStr"/>
-      <c r="I95" t="n">
-        <v>95</v>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -3871,25 +3400,18 @@
         <v>45667</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>45787</v>
+        <v>45787.99930555555</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
           <t>338 - 2012 Nissan Titan, White (5 Seats)</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
           <t>Peter Fule</t>
         </is>
-      </c>
-      <c r="I96" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="97">
@@ -3910,22 +3432,15 @@
         <v>45401</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>45402</v>
+        <v>45402.99930555555</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
           <t>338 - 2012 Nissan Titan, White (5 Seats)</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr"/>
-      <c r="I97" t="n">
-        <v>93</v>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -3945,7 +3460,7 @@
         <v>45597</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>45613</v>
+        <v>45613.99930555555</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -3958,9 +3473,6 @@
         </is>
       </c>
       <c r="H98" t="inlineStr"/>
-      <c r="I98" t="n">
-        <v>92</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -3980,7 +3492,7 @@
         <v>45594</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>45594</v>
+        <v>45594.99930555555</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -3993,9 +3505,6 @@
         </is>
       </c>
       <c r="H99" t="inlineStr"/>
-      <c r="I99" t="n">
-        <v>94</v>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -4015,22 +3524,15 @@
         <v>45561</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>45561</v>
+        <v>45561.99930555555</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
           <t>466 - 2007 Ford Expedition, Silver (7 Seats)</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
-      <c r="I100" t="n">
-        <v>107</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4050,7 +3552,7 @@
         <v>45425</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>45534</v>
+        <v>45534.99930555555</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -4063,9 +3565,6 @@
         </is>
       </c>
       <c r="H101" t="inlineStr"/>
-      <c r="I101" t="n">
-        <v>106</v>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -4085,22 +3584,15 @@
         <v>45421</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>45421</v>
+        <v>45421.99930555555</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
           <t>466 - 2007 Ford Expedition, Silver (7 Seats)</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr"/>
-      <c r="I102" t="n">
-        <v>105</v>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -4120,7 +3612,7 @@
         <v>45605</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>45605</v>
+        <v>45605.99930555555</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -4133,9 +3625,6 @@
         </is>
       </c>
       <c r="H103" t="inlineStr"/>
-      <c r="I103" t="n">
-        <v>104</v>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -4155,22 +3644,15 @@
         <v>45592</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>45594</v>
+        <v>45594.99930555555</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
           <t>466 - 2007 Ford Expedition, Silver (7 Seats)</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr"/>
-      <c r="I104" t="n">
-        <v>103</v>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -4190,22 +3672,15 @@
         <v>45401</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>45410</v>
+        <v>45410.99930555555</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
           <t>466 - 2007 Ford Expedition, Silver (7 Seats)</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
-      <c r="I105" t="n">
-        <v>108</v>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -4225,22 +3700,15 @@
         <v>45595</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>45599</v>
+        <v>45599.99930555555</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
           <t>466 - 2007 Ford Expedition, Silver (7 Seats)</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr"/>
-      <c r="I106" t="n">
-        <v>101</v>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -4260,7 +3728,7 @@
         <v>45629</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>45648</v>
+        <v>45648.99930555555</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -4276,9 +3744,6 @@
         <is>
           <t>Keven Griffen</t>
         </is>
-      </c>
-      <c r="I107" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="108">
@@ -4299,22 +3764,15 @@
         <v>45610</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>45614</v>
+        <v>45614.99930555555</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
           <t>466 - 2007 Ford Expedition, Silver (7 Seats)</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr"/>
-      <c r="I108" t="n">
-        <v>99</v>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -4334,25 +3792,18 @@
         <v>45629</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>45647</v>
+        <v>45647.99930555555</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
           <t>466 - 2007 Ford Expedition, Silver (7 Seats)</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
           <t>Keven Griffen</t>
         </is>
-      </c>
-      <c r="I109" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="110">
@@ -4373,7 +3824,7 @@
         <v>45568</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>45572</v>
+        <v>45572.99930555555</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -4386,9 +3837,6 @@
         </is>
       </c>
       <c r="H110" t="inlineStr"/>
-      <c r="I110" t="n">
-        <v>102</v>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -4408,7 +3856,7 @@
         <v>45523</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>45524</v>
+        <v>45524.99930555555</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -4421,9 +3869,6 @@
         </is>
       </c>
       <c r="H111" t="inlineStr"/>
-      <c r="I111" t="n">
-        <v>119</v>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -4443,7 +3888,7 @@
         <v>45527</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>45527</v>
+        <v>45527.99930555555</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -4456,9 +3901,6 @@
         </is>
       </c>
       <c r="H112" t="inlineStr"/>
-      <c r="I112" t="n">
-        <v>118</v>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -4478,22 +3920,15 @@
         <v>45441</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>45442</v>
+        <v>45442.99930555555</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
           <t>467 - 2011 Chevy Silverado, Pearl (5 Seats)</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
-      <c r="I113" t="n">
-        <v>117</v>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -4513,22 +3948,15 @@
         <v>45516</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>45521</v>
+        <v>45521.99930555555</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
           <t>467 - 2011 Chevy Silverado, Pearl (5 Seats)</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr"/>
-      <c r="I114" t="n">
-        <v>116</v>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -4548,7 +3976,7 @@
         <v>45533</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>45534</v>
+        <v>45534.99930555555</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -4564,9 +3992,6 @@
         <is>
           <t>Adair Patterson</t>
         </is>
-      </c>
-      <c r="I115" t="n">
-        <v>115</v>
       </c>
     </row>
     <row r="116">
@@ -4587,7 +4012,7 @@
         <v>45496</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>45506</v>
+        <v>45506.99930555555</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -4600,9 +4025,6 @@
         </is>
       </c>
       <c r="H116" t="inlineStr"/>
-      <c r="I116" t="n">
-        <v>112</v>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -4622,22 +4044,15 @@
         <v>45401</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>45402</v>
+        <v>45402.99930555555</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
           <t>467 - 2011 Chevy Silverado, Pearl (5 Seats)</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
-      <c r="I117" t="n">
-        <v>113</v>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -4657,22 +4072,15 @@
         <v>45408</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>45412</v>
+        <v>45412.99930555555</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
           <t>467 - 2011 Chevy Silverado, Pearl (5 Seats)</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr"/>
-      <c r="I118" t="n">
-        <v>111</v>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -4692,25 +4100,18 @@
         <v>45488</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>45491</v>
+        <v>45491.99930555555</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
           <t>467 - 2011 Chevy Silverado, Pearl (5 Seats)</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr">
         <is>
           <t>Shay Levine</t>
         </is>
-      </c>
-      <c r="I119" t="n">
-        <v>110</v>
       </c>
     </row>
     <row r="120">
@@ -4731,22 +4132,15 @@
         <v>45440</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>45440</v>
+        <v>45440.99930555555</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
           <t>467 - 2011 Chevy Silverado, Pearl (5 Seats)</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr"/>
-      <c r="I120" t="n">
-        <v>109</v>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -4766,7 +4160,7 @@
         <v>45478</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>45487</v>
+        <v>45487.99930555555</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -4779,9 +4173,6 @@
         </is>
       </c>
       <c r="H121" t="inlineStr"/>
-      <c r="I121" t="n">
-        <v>120</v>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -4801,22 +4192,15 @@
         <v>45509</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>45513</v>
+        <v>45513.99930555555</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
           <t>467 - 2011 Chevy Silverado, Pearl (5 Seats)</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr"/>
-      <c r="I122" t="n">
-        <v>114</v>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -4836,7 +4220,7 @@
         <v>45431</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>45436</v>
+        <v>45436.99930555555</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -4849,9 +4233,36 @@
         </is>
       </c>
       <c r="H123" t="inlineStr"/>
-      <c r="I123" t="n">
-        <v>121</v>
-      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">325 </t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Jill Beckmann</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Reserved</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="n">
+        <v>46069</v>
+      </c>
+      <c r="E124" s="2" t="n">
+        <v>46073.99930555555</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>325 - Chevy Trail Boss, White</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added entry for Salli Dymond
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H124"/>
+  <dimension ref="A1:H125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4235,10 +4235,8 @@
       <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t xml:space="preserve">325 </t>
-        </is>
+      <c r="A124" t="n">
+        <v>325</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -4263,6 +4261,44 @@
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">329 </t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Salli Dymond</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="E125" s="2" t="n">
+        <v>46076.99930555555</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>329 - Chevy Trail Boss, White</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>The vehicle will be used for a trip to Sierra Ancha for field/research purposes. I will be traveling with one other person, for a total of two occupants</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Seyed Mohammad Moein Sadeghi</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added entry for OUT OF COMMISSION
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H125"/>
+  <dimension ref="A1:H126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4263,10 +4263,8 @@
       <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t xml:space="preserve">329 </t>
-        </is>
+      <c r="A125" t="n">
+        <v>329</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -4299,6 +4297,40 @@
           <t>Seyed Mohammad Moein Sadeghi</t>
         </is>
       </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">330 </t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>OUT OF COMMISSION</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>46087.99930555555</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>330 - Toyota Camry</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>out for repairs</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added entry for Anita Joy Antoninka
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H126"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4330,6 +4330,44 @@
       </c>
       <c r="H126" t="inlineStr"/>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">330 </t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Anita Joy Antoninka</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Reserved</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>46122</v>
+      </c>
+      <c r="E127" s="2" t="n">
+        <v>46131.99930555555</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>330 - Toyota Camry</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>trip- to phoenix</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Kara Gibson</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added entry for Andi Thode
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H127"/>
+  <dimension ref="A1:H128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4331,10 +4331,8 @@
       <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">330 </t>
-        </is>
+      <c r="A127" t="n">
+        <v>330</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -4365,6 +4363,44 @@
       <c r="H127" t="inlineStr">
         <is>
           <t>Kara Gibson</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">268 </t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Andi Thode</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Reserved</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="n">
+        <v>46086</v>
+      </c>
+      <c r="E128" s="2" t="n">
+        <v>46088.99930555555</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>268 - 2017 Ford F-150, Silver(6 Seats)</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>going to Apache Junction, AZ for one week. This will be used for field work for a masters project. There are three people going.</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Regan Delaney, Caleb Smith</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated data via interactive editor
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -4367,10 +4367,8 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t xml:space="preserve">268 </t>
-        </is>
+      <c r="A128" t="n">
+        <v>268</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -4400,7 +4398,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Regan Delaney, Caleb Smith</t>
+          <t>Regan Delaney, Caleb Smith, Reagan Lind</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added entry for Nathan Saurer
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H129"/>
+  <dimension ref="A1:H130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4403,10 +4403,8 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t xml:space="preserve">321 </t>
-        </is>
+      <c r="A129" t="n">
+        <v>321</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -4439,6 +4437,40 @@
           <t>Emory Ellis</t>
         </is>
       </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>331</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Nathan Saurer</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Reserved</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="n">
+        <v>46101</v>
+      </c>
+      <c r="E130" s="2" t="n">
+        <v>46111.99930555555</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>331- 2024  Toyota Sienna Hybrid, White (8 seats)</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>We need two vehicles to help with a busy week of rentals at the Motor Pool. We have a group that needs to fit 10 bodies all with large packs.</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added entry for Richard Hofstetter
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H134"/>
+  <dimension ref="A1:H135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4563,10 +4563,8 @@
       <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">330 </t>
-        </is>
+      <c r="A134" t="n">
+        <v>330</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -4591,6 +4589,44 @@
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">310 </t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Richard Hofstetter</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="E135" s="2" t="n">
+        <v>46111.99930555555</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>310 - Chevy Trail Boss, White</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>visit OSS sites at Mogollon Rim</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Julia Totty</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added entry for Kelsey Bryant
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H136"/>
+  <dimension ref="A1:H137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4627,10 +4627,8 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">329 </t>
-        </is>
+      <c r="A136" t="n">
+        <v>329</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -4659,6 +4657,44 @@
         </is>
       </c>
       <c r="H136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">310 </t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Kelsey Bryant</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Reserved</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="n">
+        <v>46118</v>
+      </c>
+      <c r="E137" s="2" t="n">
+        <v>46119.99930555555</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>310 - Chevy Trail Boss, White</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> collect data, install equipment, perform sampling at research field site; Payson Arizona; 3 occupants</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Salli Dymond, Ari DellaSala</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added entry for Seafha Ramos
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H138"/>
+  <dimension ref="A1:H139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4714,6 +4714,44 @@
       </c>
       <c r="H138" t="inlineStr"/>
     </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>331</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Seafha Ramos</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Reserved</t>
+        </is>
+      </c>
+      <c r="D139" s="1" t="n">
+        <v>46132</v>
+      </c>
+      <c r="E139" s="1" t="n">
+        <v>46146.99930555555</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>331- 2024  Toyota Sienna Hybrid, White (8 seats)</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>NAU Mountain Campus and Environs, Tribal engagement. Anticipate 1-2 occupants</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Destiny Sanderson</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added entry for Matthew Bowker
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H139"/>
+  <dimension ref="A1:H140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4715,10 +4715,8 @@
       <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>331</t>
-        </is>
+      <c r="A139" t="n">
+        <v>331</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -4749,6 +4747,44 @@
       <c r="H139" t="inlineStr">
         <is>
           <t>Destiny Sanderson</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">268 </t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Matthew Bowker</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D140" s="1" t="n">
+        <v>46129</v>
+      </c>
+      <c r="E140" s="1" t="n">
+        <v>46129.99930555555</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>268 - 2017 Ford F-150, Silver(6 Seats)</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>We will be taking this vehicle to the preacher fire burn scar on Dimond Peak, near Payson, Arizona. 2 Occupants.</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Ella Santana-Propper</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added entry for Kristen Waring
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H142"/>
+  <dimension ref="A1:H143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4815,10 +4815,8 @@
       <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>331</t>
-        </is>
+      <c r="A142" t="n">
+        <v>331</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -4849,6 +4847,44 @@
       <c r="H142" t="inlineStr">
         <is>
           <t>Sierra Gugel</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">268 </t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Kristen Waring</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Reserved</t>
+        </is>
+      </c>
+      <c r="D143" s="1" t="n">
+        <v>46137</v>
+      </c>
+      <c r="E143" s="1" t="n">
+        <v>46138.99930555555</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>268 - 2017 Ford F-150, Silver(6 Seats)</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Travel to Mt. Elden, 4 occupants</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Abirel Acharya</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added entry for Derek Uhey
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5414,10 +5414,8 @@
       <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t xml:space="preserve">268 </t>
-        </is>
+      <c r="A160" t="n">
+        <v>268</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -5448,6 +5446,44 @@
       <c r="H160" t="inlineStr">
         <is>
           <t>Emory Ellis</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">466 </t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Derek Uhey</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D161" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E161" s="1" t="n">
+        <v>46366.99930555555</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>466 - 2007 Ford Expedition, Silver (7 Seats)</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Full semester check out</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Derek Uhey, Kelsey Bryant</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added entry for Adair Patterson
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H169"/>
+  <dimension ref="A1:H170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5726,10 +5726,8 @@
       <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t xml:space="preserve">332 </t>
-        </is>
+      <c r="A169" t="n">
+        <v>332</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -5760,6 +5758,40 @@
       <c r="H169" t="inlineStr">
         <is>
           <t>Villette Barlow, Nickolas Walker</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">333 </t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Adair Patterson</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D170" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="E170" s="1" t="n">
+        <v>46315.99930555555</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Adair Patterson</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added entry for Georgia Roberts
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H171"/>
+  <dimension ref="A1:H172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5829,6 +5829,44 @@
         </is>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">330 </t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Georgia Roberts</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D172" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E172" s="1" t="n">
+        <v>46279.99930555555</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>330 - Toyota Camry</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Georgia Roberts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>